<commit_message>
feature: red dot system 추가. refactor: GAME_TEXT string table 분리.
</commit_message>
<xml_diff>
--- a/input/Domains/Common/StringTable.xlsx
+++ b/input/Domains/Common/StringTable.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/strings/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Common/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CE444B2-462E-6A40-BAA5-3A78437AEA2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{702233DE-44E9-B34C-B4BD-9F0B88918A86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2060" yWindow="500" windowWidth="36980" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1420" yWindow="500" windowWidth="36980" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TEXT" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
   <si>
     <t>id</t>
   </si>
@@ -107,51 +107,6 @@
   </si>
   <si>
     <t>ネットワークエラー</t>
-  </si>
-  <si>
-    <t>btn_start</t>
-  </si>
-  <si>
-    <t>시작 버튼</t>
-  </si>
-  <si>
-    <t>Start</t>
-  </si>
-  <si>
-    <t>시작</t>
-  </si>
-  <si>
-    <t>開始</t>
-  </si>
-  <si>
-    <t>btn_quit</t>
-  </si>
-  <si>
-    <t>종료 버튼</t>
-  </si>
-  <si>
-    <t>Quit</t>
-  </si>
-  <si>
-    <t>종료</t>
-  </si>
-  <si>
-    <t>終了</t>
-  </si>
-  <si>
-    <t>loading</t>
-  </si>
-  <si>
-    <t>로딩 중</t>
-  </si>
-  <si>
-    <t>Loading...</t>
-  </si>
-  <si>
-    <t>로딩 중...</t>
-  </si>
-  <si>
-    <t>読み込み中...</t>
   </si>
 </sst>
 </file>
@@ -535,7 +490,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -640,62 +595,11 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
-      <c r="A7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" t="s">
-        <v>37</v>
-      </c>
-      <c r="E8" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B9" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" t="s">
-        <v>41</v>
-      </c>
-      <c r="D9" t="s">
-        <v>42</v>
-      </c>
-      <c r="E9" t="s">
-        <v>43</v>
-      </c>
-    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E9" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:E6" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>